<commit_message>
AUS-4649 Fix for sample repository batch upload creating merged keywords - Allow keywords to be separated by commas - Change separators from semi-colons to commas in the batch upload example file
</commit_message>
<xml_diff>
--- a/ckan/src/shared/public/base/files/auscope-sample-template-v3.xlsx
+++ b/ckan/src/shared/public/base/files/auscope-sample-template-v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csiroau-my.sharepoint.com/personal/faz014_csiro_au/Documents/AuScopeRepositories/DEPOSITS/TomAndrewsGSV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="13_ncr:1_{1BE9CD1B-2604-854E-8DB4-78D21EF16BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C16C3D14-F102-4608-B686-F3C38220E307}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="13_ncr:1_{1BE9CD1B-2604-854E-8DB4-78D21EF16BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE519DFC-7992-4467-BDE5-906410A097DC}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1990" windowWidth="19200" windowHeight="11690" activeTab="1" xr2:uid="{A55ED5CA-6264-7D48-B05A-EF7CBEC13C1D}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="11690" activeTab="1" xr2:uid="{A55ED5CA-6264-7D48-B05A-EF7CBEC13C1D}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="7" r:id="rId1"/>
@@ -248,9 +248,6 @@
   </si>
   <si>
     <t xml:space="preserve">Samples generated from Aircore drilling of the project MERIWA M452 </t>
-  </si>
-  <si>
-    <t>Polished Round (25mm);Lateritic &amp; supergene gold deposits</t>
   </si>
   <si>
     <t>GXAC0218-72</t>
@@ -737,6 +734,9 @@
   </si>
   <si>
     <t>QA-QC</t>
+  </si>
+  <si>
+    <t>Polished Round (25mm), Lateritic &amp; supergene gold deposits</t>
   </si>
 </sst>
 </file>
@@ -51124,13 +51124,13 @@
         <v>68</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>69</v>
+        <v>231</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G2" s="45">
         <v>44986</v>
@@ -51139,7 +51139,7 @@
         <v>45019</v>
       </c>
       <c r="K2" s="42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L2" s="50">
         <v>-28.061646378978502</v>
@@ -51151,30 +51151,30 @@
         <v>4326</v>
       </c>
       <c r="R2" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="S2" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="S2" s="46" t="s">
+      <c r="T2" s="42" t="s">
         <v>73</v>
       </c>
-      <c r="T2" s="42" t="s">
+      <c r="U2" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="U2" s="42" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A3" s="42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B3" s="42" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>69</v>
+        <v>231</v>
       </c>
       <c r="D3" s="42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G3" s="45">
         <v>44950</v>
@@ -51189,7 +51189,7 @@
         <v>172.5</v>
       </c>
       <c r="K3" s="42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L3" s="50">
         <v>-28.0616687063239</v>
@@ -51201,13 +51201,13 @@
         <v>4326</v>
       </c>
       <c r="R3" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="S3" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="S3" s="46" t="s">
-        <v>73</v>
-      </c>
       <c r="T3" s="42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -51310,68 +51310,68 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="C2" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="D2" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="E2" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="H2" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="H2" s="29" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" s="24" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" s="24" t="s">
+      <c r="B3" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="24" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="D4" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="E4" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="E3" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="24" t="s">
+      <c r="F4" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F4" s="24" t="s">
+      <c r="G4" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="G4" s="29" t="s">
+      <c r="H4" s="29" t="s">
         <v>88</v>
-      </c>
-      <c r="H4" s="29" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -51454,30 +51454,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="24" t="s">
+      <c r="D2" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="24" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" s="24" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A3" s="24" t="s">
+      <c r="B3" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="C3" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="D3" s="24" t="s">
         <v>95</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -51558,16 +51558,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>98</v>
-      </c>
       <c r="G2" s="24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -51622,571 +51622,571 @@
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="J1" s="9" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" t="s">
         <v>109</v>
       </c>
-      <c r="B2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>110</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>111</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>112</v>
       </c>
-      <c r="G2" t="s">
-        <v>113</v>
-      </c>
       <c r="H2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I2" s="4">
         <v>4202</v>
       </c>
       <c r="J2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>79</v>
+      <c r="C3" t="s">
+        <v>89</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>115</v>
       </c>
-      <c r="C3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>117</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>118</v>
       </c>
-      <c r="G3" t="s">
-        <v>119</v>
-      </c>
       <c r="H3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I3" s="4">
         <v>4203</v>
       </c>
       <c r="J3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B4" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" t="s">
         <v>121</v>
       </c>
-      <c r="D4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>122</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>123</v>
       </c>
-      <c r="G4" t="s">
-        <v>124</v>
-      </c>
       <c r="H4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I4" s="4">
         <v>4283</v>
       </c>
       <c r="J4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" t="s">
         <v>127</v>
       </c>
-      <c r="D5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E5" t="s">
-        <v>90</v>
-      </c>
-      <c r="F5" t="s">
-        <v>128</v>
-      </c>
       <c r="G5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5" s="5">
         <v>4326</v>
       </c>
       <c r="J5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>130</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>131</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>132</v>
       </c>
-      <c r="G6" t="s">
-        <v>133</v>
-      </c>
       <c r="H6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I6" s="4">
         <v>4347</v>
       </c>
       <c r="J6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B7" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" t="s">
         <v>135</v>
       </c>
-      <c r="D7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>136</v>
       </c>
-      <c r="G7" t="s">
-        <v>137</v>
-      </c>
       <c r="H7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I7" s="4">
         <v>4348</v>
       </c>
       <c r="J7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B8" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B8" t="s">
+      <c r="F8" t="s">
         <v>139</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>140</v>
       </c>
-      <c r="G8" t="s">
-        <v>141</v>
-      </c>
       <c r="H8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="I8" s="4">
         <v>4938</v>
       </c>
       <c r="J8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B9" t="s">
+        <v>142</v>
+      </c>
+      <c r="F9" t="s">
         <v>143</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>144</v>
       </c>
-      <c r="G9" t="s">
-        <v>145</v>
-      </c>
       <c r="H9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="I9" s="4">
         <v>4939</v>
       </c>
       <c r="J9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I10" s="5">
         <v>4979</v>
       </c>
       <c r="J10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F11" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>150</v>
       </c>
-      <c r="G11" t="s">
-        <v>151</v>
-      </c>
       <c r="H11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I11" s="4">
         <v>7842</v>
       </c>
       <c r="J11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F12" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>153</v>
       </c>
-      <c r="G12" t="s">
-        <v>154</v>
-      </c>
       <c r="H12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I12" s="4">
         <v>7843</v>
       </c>
       <c r="J12" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F13" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>156</v>
       </c>
-      <c r="G13" t="s">
-        <v>157</v>
-      </c>
       <c r="H13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="I13" s="4">
         <v>7844</v>
       </c>
       <c r="J13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F14" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>159</v>
       </c>
-      <c r="G14" t="s">
-        <v>160</v>
-      </c>
       <c r="H14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="I14" s="4">
         <v>9462</v>
       </c>
       <c r="J14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F15" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>162</v>
       </c>
-      <c r="G15" t="s">
-        <v>163</v>
-      </c>
       <c r="H15" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I15" s="4">
         <v>9463</v>
       </c>
       <c r="J15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="F16" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>166</v>
       </c>
-      <c r="G16" t="s">
-        <v>167</v>
-      </c>
       <c r="H16" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I16" s="4">
         <v>9464</v>
       </c>
       <c r="J16" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="17" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F17" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="17" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>169</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="18" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F18" t="s">
         <v>170</v>
       </c>
-      <c r="H17" t="s">
+      <c r="G18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H18" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F19" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" t="s">
+        <v>172</v>
+      </c>
+      <c r="H19" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="18" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F18" t="s">
-        <v>171</v>
+    <row r="20" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F20" t="s">
+        <v>174</v>
       </c>
-      <c r="G18" t="s">
-        <v>172</v>
+      <c r="G20" t="s">
+        <v>175</v>
       </c>
-      <c r="H18" t="s">
-        <v>164</v>
+      <c r="H20" t="s">
+        <v>229</v>
       </c>
     </row>
-    <row r="19" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F19" t="s">
-        <v>90</v>
+    <row r="21" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F21" t="s">
+        <v>176</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G21" t="s">
+        <v>177</v>
+      </c>
+      <c r="H21" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F22" t="s">
+        <v>179</v>
+      </c>
+      <c r="G22" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="23" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F23" t="s">
+        <v>180</v>
+      </c>
+      <c r="G23" t="s">
+        <v>181</v>
+      </c>
+      <c r="H23" t="s">
         <v>173</v>
       </c>
-      <c r="H19" t="s">
-        <v>217</v>
+    </row>
+    <row r="24" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F24" t="s">
+        <v>182</v>
       </c>
-    </row>
-    <row r="20" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F20" t="s">
-        <v>175</v>
+      <c r="G24" t="s">
+        <v>183</v>
       </c>
-      <c r="G20" t="s">
-        <v>176</v>
+      <c r="H24" t="s">
+        <v>89</v>
       </c>
-      <c r="H20" t="s">
+    </row>
+    <row r="25" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F25" t="s">
+        <v>184</v>
+      </c>
+      <c r="G25" t="s">
+        <v>185</v>
+      </c>
+      <c r="H25" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="26" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F26" t="s">
+        <v>186</v>
+      </c>
+      <c r="G26" t="s">
+        <v>187</v>
+      </c>
+      <c r="H26" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F27" t="s">
+        <v>188</v>
+      </c>
+      <c r="G27" t="s">
+        <v>189</v>
+      </c>
+      <c r="H27" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="28" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F28" t="s">
+        <v>191</v>
+      </c>
+      <c r="G28" t="s">
+        <v>192</v>
+      </c>
+      <c r="H28" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="29" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F29" t="s">
+        <v>193</v>
+      </c>
+      <c r="G29" t="s">
+        <v>194</v>
+      </c>
+      <c r="H29" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="21" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F21" t="s">
-        <v>177</v>
+    <row r="30" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F30" t="s">
+        <v>195</v>
       </c>
-      <c r="G21" t="s">
-        <v>178</v>
+      <c r="G30" t="s">
+        <v>196</v>
       </c>
-      <c r="H21" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="22" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F22" t="s">
-        <v>180</v>
-      </c>
-      <c r="G22" t="s">
-        <v>92</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="H30" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="23" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F23" t="s">
-        <v>181</v>
-      </c>
-      <c r="G23" t="s">
-        <v>182</v>
-      </c>
-      <c r="H23" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="24" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F24" t="s">
-        <v>183</v>
-      </c>
-      <c r="G24" t="s">
-        <v>184</v>
-      </c>
-      <c r="H24" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="25" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F25" t="s">
-        <v>185</v>
-      </c>
-      <c r="G25" t="s">
-        <v>186</v>
-      </c>
-      <c r="H25" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="26" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F26" t="s">
-        <v>187</v>
-      </c>
-      <c r="G26" t="s">
-        <v>188</v>
-      </c>
-      <c r="H26" t="s">
+    <row r="31" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="F31" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="27" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F27" t="s">
-        <v>189</v>
+      <c r="G31" t="s">
+        <v>199</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H31" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="32" spans="6:8" x14ac:dyDescent="0.4">
+      <c r="G32" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="33" spans="7:8" x14ac:dyDescent="0.4">
+      <c r="G33" t="s">
+        <v>202</v>
+      </c>
+      <c r="H33" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="34" spans="7:8" x14ac:dyDescent="0.4">
+      <c r="G34" t="s">
+        <v>204</v>
+      </c>
+      <c r="H34" t="s">
         <v>190</v>
       </c>
-      <c r="H27" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="28" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F28" t="s">
-        <v>192</v>
-      </c>
-      <c r="G28" t="s">
-        <v>193</v>
-      </c>
-      <c r="H28" t="s">
+    </row>
+    <row r="35" spans="7:8" x14ac:dyDescent="0.4">
+      <c r="G35" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="29" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F29" t="s">
-        <v>194</v>
-      </c>
-      <c r="G29" t="s">
-        <v>195</v>
-      </c>
-      <c r="H29" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="30" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F30" t="s">
-        <v>196</v>
-      </c>
-      <c r="G30" t="s">
-        <v>197</v>
-      </c>
-      <c r="H30" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="31" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="F31" t="s">
-        <v>199</v>
-      </c>
-      <c r="G31" t="s">
-        <v>200</v>
-      </c>
-      <c r="H31" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="32" spans="6:8" x14ac:dyDescent="0.4">
-      <c r="G32" t="s">
+      <c r="H35" t="s">
         <v>201</v>
       </c>
-      <c r="H32" t="s">
-        <v>221</v>
+    </row>
+    <row r="36" spans="7:8" x14ac:dyDescent="0.4">
+      <c r="G36" t="s">
+        <v>207</v>
       </c>
-    </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.4">
-      <c r="G33" t="s">
-        <v>203</v>
-      </c>
-      <c r="H33" t="s">
+      <c r="H36" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="34" spans="7:8" x14ac:dyDescent="0.4">
-      <c r="G34" t="s">
-        <v>205</v>
-      </c>
-      <c r="H34" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="35" spans="7:8" x14ac:dyDescent="0.4">
-      <c r="G35" t="s">
-        <v>207</v>
-      </c>
-      <c r="H35" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="36" spans="7:8" x14ac:dyDescent="0.4">
-      <c r="G36" t="s">
+    <row r="37" spans="7:8" x14ac:dyDescent="0.4">
+      <c r="G37" t="s">
         <v>208</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H37" t="s">
         <v>223</v>
-      </c>
-    </row>
-    <row r="37" spans="7:8" x14ac:dyDescent="0.4">
-      <c r="G37" t="s">
-        <v>209</v>
-      </c>
-      <c r="H37" t="s">
-        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -52199,6 +52199,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C458252014B43B48B36D6FD06F31079C" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e501afea9932b3d85ce2e954c11d415d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9357ce84-a672-4584-8ddb-e5b553dfe263" xmlns:ns3="f66f598c-5a54-48fa-b12a-3e2e658c8d92" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdedd23bd9c89529fbf7422df4b0877b" ns2:_="" ns3:_="">
     <xsd:import namespace="9357ce84-a672-4584-8ddb-e5b553dfe263"/>
@@ -52460,15 +52469,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
@@ -52520,6 +52520,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87B3A6F2-3465-444D-9356-D1CE25ED63C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58204553-233F-41DC-8714-3ECF30D686DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -52538,14 +52546,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87B3A6F2-3465-444D-9356-D1CE25ED63C4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F08071E2-18BC-4FC1-ACD4-DE3D1176D952}">
   <ds:schemaRefs>

</xml_diff>